<commit_message>
docs: per-day cost model in learning tracker (planned total ~$8.26)
- Day Cost Plan tab: every day with billed services, meter/rate,
  est. cost, cumulative total, free-tier status; total ~$8.26 with
  strict destroys; note on the ~$40-70 no-allowance equivalent
- Daily Plan tab now carries each day's estimated cost
- LEARNING_PLAN cost section aligned to the refined estimate
- outside-the-bracket items: only a custom domain (~$10-15/yr at a
  registrar) would cost outside Azure entirely - optional

Amp-Thread-ID: https://ampcode.com/threads/T-01a05297-fc2d-71c9-8b96-5c9c21d32891
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Daily Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Deployments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cost Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Destroy Ritual" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Day Cost Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Deployments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cost Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Destroy Ritual" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +45,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,8 +91,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -454,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -501,7 +507,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>$200 trial credit; expected spend $20-60; destroy same-day</t>
+          <t>$200 trial credit; planned spend ~$8-15 (see Day Cost Plan); destroy same-day</t>
         </is>
       </c>
     </row>
@@ -561,7 +567,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Day 19 (Fri Sep 19): React UI on Azure Static Web Apps, its own URL</t>
+          <t>Day 19 (Sat Sep 19): React UI on Azure Static Web Apps, its own URL</t>
         </is>
       </c>
     </row>
@@ -573,7 +579,19 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>10 tracked deployments - see 'Deployments' tab</t>
+          <t>10 tracked deployments — see 'Deployments' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Cost tab</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>'Day Cost Plan' = planned cost per day + cumulative; 'Cost Log' = what you actually spent</t>
         </is>
       </c>
     </row>
@@ -601,7 +619,7 @@
     <col width="38" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
@@ -659,7 +677,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Cost $</t>
+          <t>Cost est. $</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -722,7 +740,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
     </row>
@@ -775,7 +795,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
     </row>
@@ -828,7 +850,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="n">
+        <v>0.01</v>
+      </c>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
     </row>
@@ -881,7 +905,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="n">
+        <v>0.01</v>
+      </c>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
     </row>
@@ -934,7 +960,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
     </row>
@@ -944,12 +972,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -987,7 +1015,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="n">
+        <v>0.01</v>
+      </c>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
     </row>
@@ -997,12 +1027,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1040,7 +1070,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="n">
+        <v>0.01</v>
+      </c>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
     </row>
@@ -1093,7 +1125,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
     </row>
@@ -1146,7 +1180,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="n">
+        <v>1.2</v>
+      </c>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
     </row>
@@ -1199,7 +1235,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="n">
+        <v>1.2</v>
+      </c>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1290,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="n">
+        <v>1.2</v>
+      </c>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
     </row>
@@ -1305,7 +1345,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="n">
+        <v>1.3</v>
+      </c>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
     </row>
@@ -1315,12 +1357,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1358,7 +1400,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="n">
+        <v>1.2</v>
+      </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
     </row>
@@ -1411,7 +1455,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
     </row>
@@ -1464,7 +1510,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
     </row>
@@ -1517,7 +1565,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
     </row>
@@ -1570,7 +1620,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
     </row>
@@ -1623,7 +1675,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="n">
+        <v>0.5</v>
+      </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
     </row>
@@ -1676,7 +1730,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
     </row>
@@ -1729,7 +1785,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
     </row>
@@ -1782,7 +1840,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
     </row>
@@ -1835,7 +1895,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
     </row>
@@ -1888,7 +1950,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="n">
+        <v>0.01</v>
+      </c>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
     </row>
@@ -1941,7 +2005,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
     </row>
@@ -1994,7 +2060,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
     </row>
@@ -2047,7 +2115,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
     </row>
@@ -2100,7 +2170,9 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="n">
+        <v>0.41</v>
+      </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
     </row>
@@ -2123,6 +2195,989 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Services billed that day</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Meter / rate (approx list price)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Est. cost $</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative $</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Free-tier status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>none (local only)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Resource groups (empty)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>RGs are free; only contents bill</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Key Vault</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>$0.03 per 10,000 operations</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Operations meter only — effectively free</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Key Vault</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>$0.03 per 10,000 operations</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Operations meter only — effectively free</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Resource group via Terraform</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>state kept in local file, $0</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Key Vault via Terraform</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>$0.03 per 10,000 operations</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Operations meter only — effectively free</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Key Vault + Entra app</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>app registration free</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Operations meter only — effectively free</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>cleanup day (nothing running)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>VM B2s (24h) + public IP + 30GB disk</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>~$1.00 compute + $0.09 IP + $0.10 disk</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>VM day 2 (compose stack + image build)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>same meters</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>VM day 3 (TLS / nginx)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>same meters</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>VM day 4 (CI deploys hitting it)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>compute + egress ~$0.05</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>VM day 5 (chaos tests)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>same meters</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>VM destroyed the evening before</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>resource group deleted</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>0h</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Container Apps env + API app (mostly idle)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>~$0.000024/vCPU-s consumption</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>API + worker, brief scale-up tests</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>consumption plan, 2M requests free</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>PostgreSQL B1ms + apps</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>free tier: 750 B1ms hours + 32GB/mo</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>12-month free allowance covers it</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Load test: replicas briefly at 2-3</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>consumption plan</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1-2 h</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Static Web Apps free tier + egress</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>free tier, ~100GB bandwidth/month free</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Free tier (no charge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Revision/rollback drills on existing apps</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>no new meters</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>everything destroyed</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>AKS evening: 1 node B2ms ~8h + LB</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>~$0.083/hr node + ~$0.01/hr LB</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>8h</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>7.79</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Control plane free; you pay the node</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>App Configuration</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>free tier: 1k requests/day</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Free tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>App Insights + Log Analytics</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>first 5GB ingestion/month free</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>MBs</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>First 5GB ingestion/month free</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>pipeline reruns on existing resources</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>no new meters</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>finops sweep (nothing new)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>write-up day (DB kept only if free tier)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>B1ms beyond allowance = ~$0.41/day</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>PLANNED TOTAL</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>8.26</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Without free-account allowances the same month would cost roughly $40-70 (Postgres ~$12/mo + SWA Standard + App Insights + more VM/AKS hours).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2487,7 +3542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2543,10 +3598,14 @@
       </c>
     </row>
     <row r="40">
-      <c r="E40" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>TOTAL:</t>
         </is>
+      </c>
+      <c r="E40" s="5">
+        <f>SUM(D2:D39)</f>
+        <v/>
       </c>
       <c r="F40" s="5">
         <f>SUM(E2:E39)</f>
@@ -2558,7 +3617,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2571,56 +3630,56 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Run at the END of EVERY session. No exceptions.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>1. SCREENSHOT dashboards first (portfolio evidence)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>2. az group list -o table   -- know exactly what exists</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>3. az group delete -n learn-&lt;stage&gt;-&lt;date&gt; --yes --no-wait</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>4. Terraform days: cd infra/&lt;day&gt; &amp;&amp; terraform destroy  -- review: must list only today's resources</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>5. az resource list -o table | grep &lt;date&gt;   -- no orphaned disks/NICs/IPs</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>6. az consumption usage list --top 5 -o table   -- know today's cost</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>7. Next morning: az group list   -- nothing unexpected alive</t>
         </is>

</xml_diff>